<commit_message>
Add audit-log slot 4
</commit_message>
<xml_diff>
--- a/AI Audit Log_NguyenXuanThinh.xlsx
+++ b/AI Audit Log_NguyenXuanThinh.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FPT Chuyen Nganh\Ki 7\SWD\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FPT Chuyen Nganh\Ki 7\SWD\Github_Classroom\ai-audit-log-gonthinh7\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD13B40E-368E-494A-833D-D3FC20A2BF39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20BA0E58-E46E-4BCE-8307-EA2E50D79B46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="41">
   <si>
     <t>Ví dụ: Abstraction</t>
   </si>
@@ -147,6 +147,165 @@
   <si>
     <t>Phản hồi: Đưa ra các mô tả chi tiết về các chỉnh sửa cần thao tác.
 Kiểm chứng: Tham khảo những thao tác mà AI đưa ra.</t>
+  </si>
+  <si>
+    <t>Slot4</t>
+  </si>
+  <si>
+    <t>“Dựa trên các UC đã chỉnh sửa ở Slot3, hãy giúp tôi kiểm tra lại mối liên kết giữa Actor – Use Case – Business Rule để đảm bảo không có chức năng nào bị trùng lặp hoặc thiếu luồng xử lý. Hãy phân tích theo góc nhìn Software Design và ưu tiên tính nhất quán của hệ thống.”</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Phản hồi:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> AI phân tích các Actor và chỉ ra một số UC đang bị chồng chéo trách nhiệm, đồng thời đề xuất gom các chức năng tương tự để giảm dư thừa logic. AI cũng gợi ý bổ sung Business Rule cho các trường hợp ngoại lệ. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Quyết định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Chọn chỉnh sửa lại các UC bị overlap và thêm mô tả Business Rule cho các luồng chưa rõ ràng.</t>
+    </r>
+  </si>
+  <si>
+    <t>“Hãy review sơ đồ Use Case hiện tại của tôi theo hướng mở rộng hệ thống trong tương lai. Nếu hệ thống có thêm vai trò mới hoặc tích hợp thêm module khác thì những phần nào trong thiết kế hiện tại có thể gây khó khăn?”</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Phản hồi:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> AI chỉ ra một số Use Case đang phụ thuộc cứng vào Actor hiện tại, khiến việc mở rộng role sau này khó tái sử dụng. Đồng thời AI đề xuất tách một số UC thành nhóm độc lập hơn để tăng khả năng maintain. Quyết định: Điều chỉnh lại một số quan hệ include/extend và chuẩn hóa naming convention giữa các UC.</t>
+    </r>
+  </si>
+  <si>
+    <t>“Hãy giúp tôi xác định các chức năng có nguy cơ ảnh hưởng đến bảo mật hoặc phân quyền trong hệ thống. Dựa trên sơ đồ UC hiện tại, hãy chỉ ra các điểm cần bổ sung role validation hoặc access control.”</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Phản hồi:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> AI chỉ ra một số Use Case chưa kiểm soát rõ quyền truy cập giữa các Actor và đề xuất thêm điều kiện authorization trước khi thực hiện thao tác quan trọng. AI cũng gợi ý phân tách quyền theo nhóm chức năng. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Quyết định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Bổ sung thêm mô tả phân quyền cho các UC nhạy cảm và cập nhật lại phần đặc tả chức năng.</t>
+    </r>
+  </si>
+  <si>
+    <t>“Dựa trên toàn bộ Use Case hiện tại, hãy đề xuất cách tổ chức lại module hệ thống theo hướng dễ maintain và phù hợp với Software Design. Ưu tiên việc giảm coupling và tăng khả năng tái sử dụng component.”</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Phản hồi:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> AI đề xuất chia hệ thống thành các module riêng theo domain chức năng và khuyến nghị áp dụng layered architecture để tách biệt UI, business logic và data access. Ngoài ra AI cũng gợi ý nhóm các chức năng dùng chung thành service chung để tránh lặp code. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Quyết định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Tham khảo cấu trúc module mà AI đề xuất để chuẩn bị cho bước thiết kế kiến trúc hệ thống ở các slot tiếp theo.</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -226,7 +385,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -259,21 +418,6 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -726,7 +870,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" ht="85.5">
-      <c r="A2" s="18">
+      <c r="A2" s="13">
         <v>1</v>
       </c>
       <c r="B2" s="9" t="s">
@@ -740,7 +884,7 @@
       </c>
     </row>
     <row r="3" spans="1:4" ht="57">
-      <c r="A3" s="18">
+      <c r="A3" s="13">
         <v>2</v>
       </c>
       <c r="B3" s="9" t="s">
@@ -754,7 +898,7 @@
       </c>
     </row>
     <row r="4" spans="1:4" ht="85.5">
-      <c r="A4" s="18">
+      <c r="A4" s="13">
         <v>3</v>
       </c>
       <c r="B4" s="9" t="s">
@@ -768,7 +912,7 @@
       </c>
     </row>
     <row r="5" spans="1:4" ht="42.75">
-      <c r="A5" s="18">
+      <c r="A5" s="13">
         <v>4</v>
       </c>
       <c r="B5" s="9" t="s">
@@ -790,7 +934,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69A16565-6ACB-4DDB-B0C1-55C7722368A3}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="4.625" bestFit="1" customWidth="1"/>
@@ -817,7 +961,7 @@
       <c r="A2" s="8">
         <v>1</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="12" t="s">
         <v>17</v>
       </c>
       <c r="C2" s="10" t="s">
@@ -855,20 +999,65 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
-      <c r="A5" s="12"/>
-      <c r="B5" s="13"/>
-      <c r="C5" s="14"/>
-      <c r="D5" s="15"/>
-    </row>
-    <row r="6" spans="1:4">
-      <c r="A6" s="12"/>
-      <c r="B6" s="13"/>
-      <c r="C6" s="14"/>
-      <c r="D6" s="16"/>
+    <row r="5" spans="1:4" ht="142.5">
+      <c r="A5" s="8">
+        <v>4</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="114">
+      <c r="A6" s="8">
+        <v>5</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="114">
+      <c r="A7" s="8">
+        <v>6</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="115.5">
+      <c r="A8" s="8">
+        <v>7</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>40</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Cap nhat audit-log slot5
</commit_message>
<xml_diff>
--- a/AI Audit Log_NguyenXuanThinh.xlsx
+++ b/AI Audit Log_NguyenXuanThinh.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FPT Chuyen Nganh\Ki 7\SWD\Github_Classroom\ai-audit-log-gonthinh7\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20BA0E58-E46E-4BCE-8307-EA2E50D79B46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44D6F81E-BA6C-48A3-B64F-C47525FA2AE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="3" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="1" r:id="rId1"/>
     <sheet name="Week1" sheetId="2" r:id="rId2"/>
     <sheet name="Week2" sheetId="3" r:id="rId3"/>
-    <sheet name="Assignment 3" sheetId="4" r:id="rId4"/>
+    <sheet name="Week3" sheetId="5" r:id="rId4"/>
+    <sheet name="Assignment 3" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="52">
   <si>
     <t>Ví dụ: Abstraction</t>
   </si>
@@ -305,6 +306,230 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve"> Tham khảo cấu trúc module mà AI đề xuất để chuẩn bị cho bước thiết kế kiến trúc hệ thống ở các slot tiếp theo.</t>
+    </r>
+  </si>
+  <si>
+    <t>Slot5</t>
+  </si>
+  <si>
+    <t>“Dựa trên Use Case và business flow đã hoàn thiện ở các slot trước, hãy giúp tôi xác định các class chính cần có trong hệ thống. Hãy đóng vai Software Designer và đề xuất Class Diagram ở mức domain model, bao gồm class name, responsibility và mối liên hệ cơ bản giữa các class.”</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Phản hồi</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">: AI đề xuất danh sách các entity/domain class chính dựa trên nghiệp vụ, giải thích vai trò của từng class và xác định quan hệ association cơ bản giữa chúng. AI cũng phân biệt được class nghiệp vụ và class hỗ trợ hệ thống để tránh mô hình bị rối. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Quyết định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Chọn các class phù hợp với phạm vi dự án và loại bỏ các class không cần thiết hoặc vượt ngoài scope.</t>
+    </r>
+  </si>
+  <si>
+    <t>“Hãy kiểm tra Class Diagram hiện tại của tôi và đánh giá xem có class nào bị dư trách nhiệm hoặc vi phạm nguyên tắc thiết kế không. Hãy đề xuất chỉnh sửa theo hướng Software Design.”</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Phản hồi:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> AI phân tích trách nhiệm của từng class, chỉ ra một số class đang ôm quá nhiều logic và có dependency chưa hợp lý. AI đề xuất tách nhỏ responsibility hoặc chuyển một số xử lý sang service/helper class nhằm tăng maintainability. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Quyết định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Điều chỉnh lại cấu trúc class và phân chia lại trách nhiệm để Class Diagram rõ ràng hơn.</t>
+    </r>
+  </si>
+  <si>
+    <t>“Dựa trên Class Diagram hiện tại, hãy giúp tôi xác định đúng các relationship giữa class (association, aggregation, composition). Nếu có relationship chưa hợp lý hãy giải thích nguyên nhân và đề xuất thay thế.”</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Phản hồi:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> AI kiểm tra các mối quan hệ giữa class và giải thích lý do lựa chọn từng loại relationship. Một số quan hệ bị dùng chưa đúng được AI đề xuất đổi sang association hoặc composition để phản ánh đúng vòng đời đối tượng. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Quyết định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Cập nhật lại relationship trong sơ đồ để đúng ngữ nghĩa UML và sát với nghiệp vụ hệ thống hơn.</t>
+    </r>
+  </si>
+  <si>
+    <t>“Hãy giúp tôi bổ sung attribute và method cho các class trong Class Diagram dựa trên business logic hiện tại. Chỉ tập trung vào các thành phần cần thiết, tránh thiết kế quá dư thừa hoặc lệch khỏi Use Case.”</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Phản hồi:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> AI đề xuất các thuộc tính và phương thức cốt lõi của từng class dựa trên luồng nghiệp vụ và chức năng hệ thống. Đồng thời AI chỉ ra những method nên nằm ở class nào để đảm bảo tính cohesion. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Quyết định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Chọn giữ lại các attribute/method phục vụ trực tiếp Use Case và loại bỏ các phần chưa cần thiết trong phạm vi đồ án.</t>
+    </r>
+  </si>
+  <si>
+    <t>“Hãy review tổng thể Class Diagram của tôi theo góc nhìn Software Design và khả năng mở rộng hệ thống. Nếu trong tương lai thêm chức năng hoặc actor mới thì cấu trúc class hiện tại có điểm nào dễ gây khó maintain hoặc mở rộng không?”</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Phản hồi:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> AI đánh giá mức độ mở rộng của sơ đồ class, phát hiện một số dependency có nguy cơ làm hệ thống khó scale hoặc tái sử dụng. AI đề xuất chuẩn hóa abstraction, giảm coupling giữa các class và tổ chức lại dependency để tăng extensibility. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Quyết định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Tham khảo các đề xuất của AI để chỉnh sửa Class Diagram trước khi chuyển sang thiết kế chi tiết hoặc implementation.</t>
     </r>
   </si>
 </sst>
@@ -1062,6 +1287,121 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7387A159-7646-416C-AA67-43DB3840410A}">
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="4.625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="51.875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="15">
+      <c r="A1" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="156.75">
+      <c r="A2" s="8">
+        <v>1</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="116.25">
+      <c r="A3" s="8">
+        <v>2</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="114">
+      <c r="A4" s="8">
+        <v>3</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="142.5">
+      <c r="A5" s="8">
+        <v>4</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="115.5">
+      <c r="A6" s="8">
+        <v>5</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="129.75">
+      <c r="A7" s="8">
+        <v>6</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>51</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{323516A4-AE23-41CF-AD84-97A6064FC5FB}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.25"/>

</xml_diff>

<commit_message>
Add AI Audit Log slot6
</commit_message>
<xml_diff>
--- a/AI Audit Log_NguyenXuanThinh.xlsx
+++ b/AI Audit Log_NguyenXuanThinh.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FPT Chuyen Nganh\Ki 7\SWD\Github_Classroom\ai-audit-log-gonthinh7\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44D6F81E-BA6C-48A3-B64F-C47525FA2AE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDC8F62F-448E-4E6F-BD77-6BAA6CAF3A93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="3" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="63">
   <si>
     <t>Ví dụ: Abstraction</t>
   </si>
@@ -530,6 +530,228 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve"> Tham khảo các đề xuất của AI để chỉnh sửa Class Diagram trước khi chuyển sang thiết kế chi tiết hoặc implementation.</t>
+    </r>
+  </si>
+  <si>
+    <t>Slot6</t>
+  </si>
+  <si>
+    <t>"“Dựa trên Use Case Diagram và Class Diagram hiện tại, hãy kiểm tra tính nhất quán giữa chức năng hệ thống và cấu trúc class. Mỗi Use Case có đang được hỗ trợ bởi class phù hợp hay còn thiếu mapping nào không? Hãy phân tích theo góc nhìn Software Design.”"</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Phản hồi</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">: AI đối chiếu Use Case với các class hiện tại và phát hiện một số chức năng chưa được phản ánh rõ trong Class Diagram hoặc đang bị gộp trách nhiệm chưa hợp lý. AI đề xuất bổ sung hoặc điều chỉnh class để phản ánh đúng business flow.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Quyết định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Kiểm tra lại sự liên kết giữa Use Case và Class Diagram, chỉnh sửa các class chưa phản ánh đúng nghiệp vụ.</t>
+    </r>
+  </si>
+  <si>
+    <t>“Hãy review Class Diagram của tôi để đánh giá mức độ phù hợp với các Use Case hiện tại. Kiểm tra xem có method hoặc attribute nào không phục vụ trực tiếp business logic hoặc bị thiếu đối với chức năng hệ thống không.”</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Phản hồi:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> AI đánh giá lại attribute và method của từng class, chỉ ra một số thành phần chưa gắn với Use Case cụ thể hoặc còn thiếu thao tác cần thiết cho flow xử lý. AI đề xuất tinh gọn class để tăng cohesion. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Quyết định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Giữ lại các thành phần phục vụ trực tiếp nghiệp vụ và loại bỏ các thuộc tính/method chưa cần thiết trong phạm vi hệ thống.</t>
+    </r>
+  </si>
+  <si>
+    <t>“Dựa trên sơ đồ Use Case và Class Diagram hiện tại, hãy kiểm tra lại các relationship giữa class để đảm bảo phản ánh đúng dependency của hệ thống. Nếu có quan hệ chưa đúng semantic UML hãy giải thích và đề xuất chỉnh sửa.”</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Phản hồi:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> AI rà soát các association, aggregation, composition và dependency giữa các class, đồng thời chỉ ra một số relationship đang mô tả chưa đúng bản chất nghiệp vụ. AI đề xuất điều chỉnh nhằm tăng tính rõ ràng của mô hình thiết kế. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Quyết định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Chỉnh sửa lại các relationship chưa hợp lý để đảm bảo đúng chuẩn UML và logic hệ thống.</t>
+    </r>
+  </si>
+  <si>
+    <t>“Hãy đánh giá khả năng maintain và mở rộng của Class Diagram hiện tại theo góc nhìn Software Design. Nếu trong tương lai có thêm Use Case hoặc Actor mới thì những class nào có nguy cơ coupling cao hoặc khó tái sử dụng?”</t>
+  </si>
+  <si>
+    <t>“Hãy review tổng thể sự liên kết giữa Use Case Diagram và Class Diagram của hệ thống, đảm bảo thiết kế không bị lệch với business requirement và phù hợp với nguyên tắc Software Design.”</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Phản hồi:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> AI xác định các class có dependency cao hoặc đang ôm quá nhiều trách nhiệm, từ đó đề xuất chuẩn hóa abstraction và giảm coupling nhằm tăng extensibility của hệ thống. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Quyết định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Ghi nhận các điểm có nguy cơ ảnh hưởng đến maintainability để tinh chỉnh sơ đồ class theo hướng modular hơn.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Phản hồi:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> AI tổng hợp các điểm mạnh và điểm cần chỉnh sửa trong mô hình thiết kế, đồng thời kiểm tra tính đồng nhất giữa yêu cầu chức năng và implementation model. AI đề xuất một số điều chỉnh nhỏ để tăng consistency giữa các thành phần.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Quyết định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Tham khảo phản hồi để hoàn thiện phiên bản cuối của Use Case và Class Diagram trước khi chuyển sang các bước thiết kế hoặc implementation tiếp theo.</t>
     </r>
   </si>
 </sst>
@@ -1288,7 +1510,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7387A159-7646-416C-AA67-43DB3840410A}">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="4.625" bestFit="1" customWidth="1"/>
@@ -1393,6 +1615,76 @@
       </c>
       <c r="D7" s="11" t="s">
         <v>51</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="142.5">
+      <c r="A8" s="8">
+        <v>7</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="128.25">
+      <c r="A9" s="8">
+        <v>8</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="114">
+      <c r="A10" s="8">
+        <v>9</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="D10" s="11" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="128.25">
+      <c r="A11" s="8">
+        <v>10</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="115.5">
+      <c r="A12" s="8">
+        <v>11</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add AI Audit Log Slot 7 - Slot 8
</commit_message>
<xml_diff>
--- a/AI Audit Log_NguyenXuanThinh.xlsx
+++ b/AI Audit Log_NguyenXuanThinh.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FPT Chuyen Nganh\Ki 7\SWD\Github_Classroom\ai-audit-log-gonthinh7\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDC8F62F-448E-4E6F-BD77-6BAA6CAF3A93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA49980C-4AE5-4FCE-8842-AE428EA432C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="3" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="4" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="1" r:id="rId1"/>
     <sheet name="Week1" sheetId="2" r:id="rId2"/>
     <sheet name="Week2" sheetId="3" r:id="rId3"/>
     <sheet name="Week3" sheetId="5" r:id="rId4"/>
-    <sheet name="Assignment 3" sheetId="4" r:id="rId5"/>
+    <sheet name="Week4" sheetId="6" r:id="rId5"/>
+    <sheet name="Assignment 3" sheetId="4" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="81">
   <si>
     <t>Ví dụ: Abstraction</t>
   </si>
@@ -752,6 +753,364 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve"> Tham khảo phản hồi để hoàn thiện phiên bản cuối của Use Case và Class Diagram trước khi chuyển sang các bước thiết kế hoặc implementation tiếp theo.</t>
+    </r>
+  </si>
+  <si>
+    <t>Slot7</t>
+  </si>
+  <si>
+    <t>Slot8</t>
+  </si>
+  <si>
+    <t>“Dựa trên Use Case và Class Diagram hiện tại, hãy xác định các đối tượng (objects) tham gia vào từng luồng nghiệp vụ chính. Hãy phân tích vai trò của từng object trong quá trình xử lý để chuẩn bị cho Sequence Diagram.”</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Phản hồi:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> AI xác định các actor, boundary, control và entity object tham gia trong từng use case. Đồng thời giải thích trách nhiệm của từng đối tượng trong quá trình tương tác. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Quyết định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Chọn các object cần thiết để xây dựng Sequence Diagram, tránh đưa quá nhiều thành phần không liên quan vào sơ đồ.</t>
+    </r>
+  </si>
+  <si>
+    <t>“Hãy mô tả chi tiết luồng trao đổi thông điệp (message flow) giữa các object trong Use Case quan trọng nhất của hệ thống. Chỉ rõ thứ tự xử lý và kết quả của từng bước.”</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Phản hồi:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> AI mô tả trình tự gửi và nhận message giữa các object theo từng bước nghiệp vụ. AI cũng chỉ ra các bước validation và xử lý dữ liệu cần được thể hiện trong Sequence Diagram. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Quyết định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Sử dụng luồng xử lý được đề xuất làm cơ sở để xây dựng sơ đồ tương tác.</t>
+    </r>
+  </si>
+  <si>
+    <t>“Hãy kiểm tra xem các method trong Class Diagram hiện tại đã đủ để hỗ trợ các tương tác giữa object hay chưa. Nếu thiếu method hoặc operation nào hãy đề xuất bổ sung.”</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Phản hồi:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> AI đối chiếu message flow với các method hiện có trong Class Diagram và phát hiện một số operation còn thiếu hoặc chưa được định nghĩa rõ ràng. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Quyết định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Bổ sung các operation cần thiết để đảm bảo Sequence Diagram và Class Diagram nhất quán với nhau.</t>
+    </r>
+  </si>
+  <si>
+    <t>“Dựa trên luồng nghiệp vụ hiện tại, hãy xác định các trường hợp ngoại lệ (alternative flow và exception flow) cần được thể hiện trong Sequence Diagram.”</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Phản hồi:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> AI chỉ ra các tình huống lỗi, dữ liệu không hợp lệ hoặc điều kiện đặc biệt có thể xảy ra trong quá trình xử lý. AI đề xuất sử dụng alt/opt fragment trong UML Sequence Diagram. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Quyết định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Bổ sung các luồng ngoại lệ quan trọng vào thiết kế để mô hình hóa đầy đủ nghiệp vụ hệ thống.</t>
+    </r>
+  </si>
+  <si>
+    <t>“Dựa trên Use Case, Class Diagram và message flow đã xác định, hãy hỗ trợ tôi xây dựng Sequence Diagram cho chức năng chính của hệ thống theo chuẩn UML.”</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Phản hồi:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> AI đề xuất các lifeline, activation và thứ tự message giữa các đối tượng. AI trình bày luồng xử lý theo đúng thứ tự thời gian của nghiệp vụ. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Quyết định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Sử dụng cấu trúc Sequence Diagram do AI đề xuất để hoàn thiện sơ đồ UML.</t>
+    </r>
+  </si>
+  <si>
+    <t>“Hãy kiểm tra Sequence Diagram hiện tại và đánh giá xem luồng tương tác có phản ánh đúng Use Case và Class Diagram hay không. Chỉ ra các điểm chưa nhất quán nếu có.”</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Phản hồi</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">: AI rà soát các message và operation trong Sequence Diagram, phát hiện một số bước xử lý chưa khớp với Use Case hoặc chưa tồn tại trong Class Diagram. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Quyết định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Điều chỉnh lại message flow và cập nhật các operation cần thiết để đảm bảo tính nhất quán.</t>
+    </r>
+  </si>
+  <si>
+    <t>“Hãy review Sequence Diagram dưới góc nhìn Software Design. Kiểm tra xem có object nào đang đảm nhận quá nhiều trách nhiệm hoặc tồn tại dependency không cần thiết hay không.”</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Phản hồi:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> AI đánh giá mức độ coupling giữa các đối tượng và xác định các thành phần đang xử lý quá nhiều logic nghiệp vụ. AI đề xuất phân bổ lại trách nhiệm giữa các lớp. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Quyết định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Tinh chỉnh lại thiết kế nhằm cải thiện maintainability và tuân thủ nguyên tắc phân chia trách nhiệm.</t>
+    </r>
+  </si>
+  <si>
+    <t>“Hãy đánh giá tổng thể sự liên kết giữa Use Case Diagram, Class Diagram và Sequence Diagram của hệ thống. Kiểm tra xem các mô hình UML đã phản ánh nhất quán yêu cầu nghiệp vụ và thiết kế phần mềm hay chưa.”</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Phản hồi:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> AI thực hiện đối chiếu giữa ba loại sơ đồ UML, xác nhận các thành phần chính đã được liên kết hợp lý và chỉ ra một số điểm cần chuẩn hóa thêm. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Quyết định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Hoàn thiện phiên bản cuối của các sơ đồ UML trước khi chuyển sang giai đoạn triển khai hoặc coding.</t>
     </r>
   </si>
 </sst>
@@ -1694,6 +2053,150 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02EF8BDF-27CA-4063-A9B6-B29FEC78FD31}">
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="4.625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="51.875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="15">
+      <c r="A1" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="114">
+      <c r="A2" s="8">
+        <v>1</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="101.25">
+      <c r="A3" s="8">
+        <v>2</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="99.75">
+      <c r="A4" s="8">
+        <v>3</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="101.25">
+      <c r="A5" s="8">
+        <v>4</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="87">
+      <c r="A6" s="8">
+        <v>5</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="99.75">
+      <c r="A7" s="8">
+        <v>6</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="99.75">
+      <c r="A8" s="8">
+        <v>7</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="114">
+      <c r="A9" s="8">
+        <v>8</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>80</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{323516A4-AE23-41CF-AD84-97A6064FC5FB}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.25"/>

</xml_diff>